<commit_message>
dev/small refactor of data formats
</commit_message>
<xml_diff>
--- a/test/test.xlsx
+++ b/test/test.xlsx
@@ -436,37 +436,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BOND_RETAIL_FIXED_RATE</t>
+          <t>Akcje - cały świat</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AssetType.BOND</t>
+          <t>AssetType.ETF</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8534.290000000001</v>
+        <v>14758.87066420419</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOND_RETAIL_FIXED_RATE</t>
+          <t>Obligacje skarbowe indeksowane inflacją</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AssetType.ETF</t>
+          <t>AssetType.BOND</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4621.72802</v>
+        <v>17716.67</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOND_RETAIL_INFLATION_LINKED</t>
+          <t>Obligacje skarbowe indeksowane stopą referencyjną</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -475,52 +475,52 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17716.67</v>
+        <v>8508.450000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOND_RETAIL_INTEREST_LINKED</t>
+          <t>Obligacje skarbowe o stopie stałej</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AssetType.BOND</t>
+          <t>AssetType.ETF</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8508.450000000001</v>
+        <v>4621.72802</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COMMODITY_GOLD</t>
+          <t>Obligacje skarbowe o stopie stałej</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AssetType.ETC</t>
+          <t>AssetType.BOND</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10163.76952496106</v>
+        <v>8534.290000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EQUITY_GLOBAL</t>
+          <t>Surowce - złoto</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AssetType.ETF</t>
+          <t>AssetType.ETC</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14758.87066420419</v>
+        <v>10163.76952496106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>